<commit_message>
Confirmed all 50 test cases are populated and updated submission
</commit_message>
<xml_diff>
--- a/IT23290624_Assignment 1 - Test cases.xlsx
+++ b/IT23290624_Assignment 1 - Test cases.xlsx
@@ -483,7 +483,11 @@
           <t>ඔයාට කොහොමද?</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: oyaata kohmd?</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -521,6 +525,11 @@
           <t>කොහොමද මේ වැඩේ?</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: khmda me wede?</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>UI Error</t>
@@ -600,6 +609,11 @@
           <t>මෙතනින් යන්න.</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: methnin yanna.</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>UI Error</t>
@@ -721,6 +735,11 @@
           <t>මට උදව්වක් දෙන්නකෝ</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: mata help ekk dnnko</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>UI Error</t>
@@ -758,6 +777,11 @@
           <t>පෑනක් දෙන්න පුළුවන්ද</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: pen ekk dnn pluwnd</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>UI Error</t>
@@ -837,6 +861,16 @@
           <t>එපා මචන් එපා</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: epa mchan epa</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Responses</t>
@@ -869,6 +903,16 @@
           <t>හිනා හිනා වෙනවා</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: hina hina wenawa</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>Repeated Words</t>
@@ -901,6 +945,16 @@
           <t>යන්නම යන්නම ඕනේ</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: yannama yannama one</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>Repeated Words</t>
@@ -933,6 +987,16 @@
           <t>අයියෝ... මොකක්ද මේ??</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: aiyo... mkkda me??</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Inputs with Punctuation Marks</t>
@@ -965,6 +1029,16 @@
           <t>කෝ? තාම නෑ!</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: ko? thama na!</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>Inputs with Punctuation Marks</t>
@@ -997,6 +1071,16 @@
           <t>මම යන්නම්</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: man yanm</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>Romanization / Spelling Variants</t>
@@ -1029,6 +1113,16 @@
           <t>අපි යමු</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: api ymu</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>Romanization / Spelling Variants</t>
@@ -1061,6 +1155,16 @@
           <t>ඔයා result බැලුවද?</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: oya result baluwada?</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>Isolated English Word Insertions in Singlish</t>
@@ -1093,6 +1197,16 @@
           <t>මෙවා free දෙනවා</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: meva free denava</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>Isolated English Word Insertions in Singlish</t>
@@ -1125,6 +1239,16 @@
           <t>අපි කතා කරමු after the class</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: api katha karamu after the class</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>Multi-Word English Phrases in Singlish</t>
@@ -1157,6 +1281,16 @@
           <t>මට කියන්න how to do this</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: mata kiyanna how to do this</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>Multi-Word English Phrases in Singlish</t>
@@ -1189,6 +1323,16 @@
           <t>මට mail එකක් දාන්න</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: mata mail ekk danna</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>English Digital Terms in Singlish</t>
@@ -1221,6 +1365,16 @@
           <t>download කරලා තියන්න</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: download karala thiyanna</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>English Digital Terms in Singlish</t>
@@ -1253,6 +1407,16 @@
           <t>facebook එකේ තිබ්බා</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: facebook eke thibba</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>Platform/App Names in Singlish</t>
@@ -1285,6 +1449,16 @@
           <t>insta දාපන් මචන්</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: insta dapan mchan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>Platform/App Names in Singlish</t>
@@ -1317,6 +1491,16 @@
           <t>NIC එක පෙන්වන්න</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: NIC eka pennanna</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>English Abbreviations/Acronyms in Singlish</t>
@@ -1349,6 +1533,16 @@
           <t>USA වලට ගියා</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: USA walata giya</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>English Abbreviations/Acronyms in Singlish</t>
@@ -1381,6 +1575,16 @@
           <t>exam එක කවදාද?</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: exam eka kawadda?</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
           <t>English Clipped Forms in Singlish</t>
@@ -1413,6 +1617,16 @@
           <t>uni යන්න දවසක් නෑ</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: uni yanna dawasak na</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>English Clipped Forms in Singlish</t>
@@ -1445,6 +1659,16 @@
           <t>Colombo වලට යමු</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: Colombo walata yamu</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>Place Names Embedded in Singlish</t>
@@ -1477,6 +1701,16 @@
           <t>Kandy කතා හිතෙනවා</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: Kandy katha hithenawa</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>Place Names Embedded in Singlish</t>
@@ -1509,6 +1743,16 @@
           <t>Amal කන්ද ගිහින්</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: Amal kanda gihin</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>Person Names Embedded in Singlish</t>
@@ -1541,6 +1785,16 @@
           <t>Sunil අයියා ආවා</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: Sunil ayya awa</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
           <t>Person Names Embedded in Singlish</t>
@@ -1573,6 +1827,16 @@
           <t>100ක් දුන්නද?</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: 100k dunnada?</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
           <t>Inputs with Numbers and Numeric Suffixes</t>
@@ -1605,6 +1869,16 @@
           <t>2nd දවස වෙනකන්</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: 2nd dawasa wenakan</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>Inputs with Numbers and Numeric Suffixes</t>
@@ -1637,6 +1911,16 @@
           <t>Rs. 1000 වගේ වෙයි</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: Rs. 1000 wage wei</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr">
         <is>
           <t>Inputs with Currency</t>
@@ -1669,6 +1953,16 @@
           <t>500 LKR ගෙවන්න</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: 500 LKR gewanna</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr">
         <is>
           <t>Inputs with Currency</t>
@@ -1701,6 +1995,16 @@
           <t>9:00 AM වෙනකන් එන්න</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: 9:00 AM wenakan enna</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
           <t>Inputs with Time Formats</t>
@@ -1733,6 +2037,16 @@
           <t>රෑ 10pm ට වගේ</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: re 10pm ta wage</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
           <t>Inputs with Time Formats</t>
@@ -1765,6 +2079,16 @@
           <t>2026/05/04 දවස</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: 2026/05/04 davasa</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
           <t>Inputs with Dates</t>
@@ -1797,6 +2121,16 @@
           <t>May 5 වෙනිදා</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: May 5 wenidha</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
           <t>Inputs with Dates</t>
@@ -1829,6 +2163,16 @@
           <t>10kg තියනවාද?</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: 10kg thiyanawada?</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr">
         <is>
           <t>Inputs with Unit of Measurements</t>
@@ -1861,6 +2205,16 @@
           <t>අඩි 5ක් විතර</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: adi 5k withara</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr">
         <is>
           <t>Inputs with Unit of Measurements</t>
@@ -1893,6 +2247,16 @@
           <t>සිරාවටම එලකිරි</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: sirawatama elakiri</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr">
         <is>
           <t>Inputs with Slang and Casual Phrasing</t>
@@ -1925,6 +2289,16 @@
           <t>ලොවෙත් නෑ මචන්</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: loweth na mchan</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr">
         <is>
           <t>Inputs with Slang and Casual Phrasing</t>
@@ -1957,6 +2331,16 @@
           <t>check test.com</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: check test.com</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G46" t="inlineStr">
         <is>
           <t>Online Indentifiers in Singlish</t>
@@ -1989,6 +2373,16 @@
           <t>email: x@y.com</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: email: x@y.com</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr">
         <is>
           <t>Online Indentifiers in Singlish</t>
@@ -2021,6 +2415,16 @@
           <t>පට්ට 🚀</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: patta 🚀</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr">
         <is>
           <t>Inputs Containing Emojis</t>
@@ -2053,6 +2457,16 @@
           <t>දුකයි 😢</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: dukai 😢</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr">
         <is>
           <t>Inputs Containing Emojis</t>
@@ -2085,6 +2499,16 @@
           <t>මේ මොකක්ද මචන් ඔයා කරන්නේ? පස්සේ බලමු.</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: me mkkada mchan oya krnne? pahuwela balamu.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr">
         <is>
           <t>Question forms</t>
@@ -2115,6 +2539,16 @@
       <c r="D51" t="inlineStr">
         <is>
           <t>මට මේක පොඩ්ඩක් කියලා දෙන්නකෝ. මචන් ඔයා කොහෙද ඉන්නේ? මම හෙට office එන්නම්. එතකොට උදව්වක් දෙන්න පුළුවන්ද? thanks මචන්. එලකිරි!</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Incorrect transliteration for: mata meka poddak kiyala dennako. mchan oya koheda inne? mama heta office ennam. ethakota help ekk dnn puluwanda? thanks mchan. elakiri!</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">

</xml_diff>